<commit_message>
Update authenticator description in FSH profile 4d0ad92feada57435b87b161615552c4a2197e30
</commit_message>
<xml_diff>
--- a/nriss-patch-2/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nriss-patch-2/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-02-24T15:04:42+00:00</t>
+    <t>2026-04-22T16:14:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1026,7 +1026,7 @@
 </t>
   </si>
   <si>
-    <t>Cet attribut représente l’acteur validant le document et prenant la responsabilité du contenu médical de celui-ci. Il peut s’agir de l’auteur du document si celui-ci est une personne et s’il endosse la responsabilité du contenu médical de ses documents. Si l’auteur est un dispositif, cet attribut doit représenter la personne responsable de l’action effectuée par le dispositif. Pour les documents d’expression personnelle du patient, cet attribut fait référence au patient.</t>
+    <t>Cet attribut représente l’acteur validant le document et prenant la responsabilité du contenu médical de celui-ci. Il peut s’agir de l’auteur du document si celui-ci est une personne et s’il endosse la responsabilité du contenu médical de ses documents. Si l’auteur est un dispositif, cet attribut doit représenter l'organisation responsable de l’action effectuée par le dispositif. Dans le cas où le document est poussé par le patient, l'authenticator doit rester vide.</t>
   </si>
   <si>
     <t>Which person or organization authenticates that this document is valid.</t>

</xml_diff>

<commit_message>
align simplifiedpublish et comprehensivedocumentreference c227178af20538d5cd1f26ef377eaf3d53f5bc77
</commit_message>
<xml_diff>
--- a/nriss-patch-2/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
+++ b/nriss-patch-2/ig/StructureDefinition-pdsm-comprehensive-document-reference.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-22T16:17:14+00:00</t>
+    <t>2026-05-27T14:01:46+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1026,7 +1026,7 @@
 </t>
   </si>
   <si>
-    <t>Cet attribut représente l’acteur validant le document et prenant la responsabilité du contenu médical de celui-ci. Il peut s’agir de l’auteur du document si celui-ci est une personne et s’il endosse la responsabilité du contenu médical de ses documents. Si l’auteur est un dispositif, cet attribut doit représenter l'organisation responsable de l’action effectuée par le dispositif. L'authenticator DOIT être renseigné, sauf dans le cas où le document est une expression personnelle du patient, auquel cas l'authenticator doit rester vide.</t>
+    <t>Cet attribut représente l’acteur validant le document et prenant la responsabilité du contenu médical de celui-ci. Il peut s’agir de l’auteur du document si celui-ci est une personne et s’il endosse la responsabilité du contenu médical de ses documents.</t>
   </si>
   <si>
     <t>Which person or organization authenticates that this document is valid.</t>

</xml_diff>